<commit_message>
Slides & Session 2
</commit_message>
<xml_diff>
--- a/_data/sessions.xlsx
+++ b/_data/sessions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Github/jirelations/25christentum/_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E62DC8-35AB-8647-ADEB-1743413A55C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEFAF54-203F-1840-8276-F68554D46808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -241,7 +241,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="91">
   <si>
     <t>blank</t>
   </si>
@@ -500,6 +500,21 @@
   </si>
   <si>
     <t xml:space="preserve">Das Datum des nächsten Ostern nach den Quartodecimans bzw. nach Aphrahats Vorgaben rechnen. </t>
+  </si>
+  <si>
+    <t>slide-frontmatter</t>
+  </si>
+  <si>
+    <t>slide-body1</t>
+  </si>
+  <si>
+    <t>slide-body2</t>
+  </si>
+  <si>
+    <t>slide-content</t>
+  </si>
+  <si>
+    <t>slide-filename</t>
   </si>
 </sst>
 </file>
@@ -614,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -656,6 +671,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -962,7 +980,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" hidden="1" customWidth="1"/>
@@ -980,10 +998,11 @@
     <col min="13" max="13" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="77.83203125" customWidth="1"/>
     <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.5" customWidth="1"/>
+    <col min="17" max="18" width="32.5" customWidth="1"/>
+    <col min="19" max="19" width="39.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1035,8 +1054,23 @@
       <c r="Q1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="R1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="S1" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="T1" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="U1" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="V1" s="19" t="s">
+        <v>89</v>
+      </c>
     </row>
-    <row r="2" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="3">
         <v>1</v>
       </c>
@@ -1093,8 +1127,105 @@
 level: overview
 ---</v>
       </c>
+      <c r="R2" t="str">
+        <f>_xlfn.REGEXREPLACE(D2,"\.md","-slides.md")</f>
+        <v>2025-04-28-1-slides.md</v>
+      </c>
+      <c r="S2" t="str">
+        <f>"---
+layout: reveal
+title: '"&amp;G2&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B2&amp;"
+tags: ["&amp;B2&amp;",slides]
+category: slides
+image: "&amp;K2&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K2&amp;"'
+---
+"</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Ist das Christentum eine westliche Religion?'
+author: 'Nathan Gibson'
+session: 1
+tags: [1,slides]
+category: slides
+image: good-friday-aleppo.jpg
+parallaxBackgroundImage: 'assets/img/good-friday-aleppo.jpg'
+---
+</v>
+      </c>
+      <c r="T2" t="str">
+        <f>"# Einführung ins Christentum
+{: .r-fit-text}
+### "&amp;G2&amp;"
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+"&amp;N1&amp;"
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+"&amp;N2</f>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Ist das Christentum eine westliche Religion?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+objective
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+1. Eigene Ziele im Kurs setzen.
+2. Westliche Vorstellungen des Christentums erstmal hinterfragen.</v>
+      </c>
+      <c r="U2" t="str">
+        <f>"
+## Lektüre
+## Diskussion
+## Vorschau
+"&amp;G3</f>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie wird die christliche Botschaft idealerweise vermittelt?</v>
+      </c>
+      <c r="V2" t="str">
+        <f>_xlfn.CONCAT(S2:U2)</f>
+        <v>---
+layout: reveal
+title: 'Ist das Christentum eine westliche Religion?'
+author: 'Nathan Gibson'
+session: 1
+tags: [1,slides]
+category: slides
+image: good-friday-aleppo.jpg
+parallaxBackgroundImage: 'assets/img/good-friday-aleppo.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Ist das Christentum eine westliche Religion?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+objective
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+1. Eigene Ziele im Kurs setzen.
+2. Westliche Vorstellungen des Christentums erstmal hinterfragen.
+## Lektüre
+## Diskussion
+## Vorschau
+Wie wird die christliche Botschaft idealerweise vermittelt?</v>
+      </c>
     </row>
-    <row r="3" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3">
         <v>2</v>
       </c>
@@ -1154,8 +1285,105 @@
 level: overview
 ---</v>
       </c>
+      <c r="R3" t="str">
+        <f t="shared" ref="R3:R14" si="6">_xlfn.REGEXREPLACE(D3,"\.md","-slides.md")</f>
+        <v>2025-05-05-2-slides.md</v>
+      </c>
+      <c r="S3" t="str">
+        <f t="shared" ref="S3:S14" si="7">"---
+layout: reveal
+title: '"&amp;G3&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B3&amp;"
+tags: ["&amp;B3&amp;",slides]
+category: slides
+image: "&amp;K3&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K3&amp;"'
+---
+"</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie wird die christliche Botschaft idealerweise vermittelt?'
+author: 'Nathan Gibson'
+session: 2
+tags: [2,slides]
+category: slides
+image: ihlara-valley-cappadocia.jpg
+parallaxBackgroundImage: 'assets/img/ihlara-valley-cappadocia.jpg'
+---
+</v>
+      </c>
+      <c r="T3" t="str">
+        <f t="shared" ref="T3:T14" si="8">"# Einführung ins Christentum
+{: .r-fit-text}
+### "&amp;G3&amp;"
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+"&amp;N2&amp;"
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+"&amp;N3</f>
+        <v xml:space="preserve"># Einführung ins Christentum
+{: .r-fit-text}
+### Wie wird die christliche Botschaft idealerweise vermittelt?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+1. Eigene Ziele im Kurs setzen.
+2. Westliche Vorstellungen des Christentums erstmal hinterfragen.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Die Rolle der schriftlichen und mündlichen "apostolischen" Traditionen im frühchristlichen Selbstverständnis skizzieren können. </v>
+      </c>
+      <c r="U3" t="str">
+        <f t="shared" ref="U3:U14" si="9">"
+## Lektüre
+## Diskussion
+## Vorschau
+"&amp;G4</f>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Was wird mit wem gefeiert?</v>
+      </c>
+      <c r="V3" t="str">
+        <f t="shared" ref="V3:V14" si="10">_xlfn.CONCAT(S3:U3)</f>
+        <v>---
+layout: reveal
+title: 'Wie wird die christliche Botschaft idealerweise vermittelt?'
+author: 'Nathan Gibson'
+session: 2
+tags: [2,slides]
+category: slides
+image: ihlara-valley-cappadocia.jpg
+parallaxBackgroundImage: 'assets/img/ihlara-valley-cappadocia.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie wird die christliche Botschaft idealerweise vermittelt?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+1. Eigene Ziele im Kurs setzen.
+2. Westliche Vorstellungen des Christentums erstmal hinterfragen.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Die Rolle der schriftlichen und mündlichen "apostolischen" Traditionen im frühchristlichen Selbstverständnis skizzieren können. 
+## Lektüre
+## Diskussion
+## Vorschau
+Was wird mit wem gefeiert?</v>
+      </c>
     </row>
-    <row r="4" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3">
         <v>3</v>
       </c>
@@ -1215,8 +1443,78 @@
 level: overview
 ---</v>
       </c>
+      <c r="R4" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-05-12-3-slides.md</v>
+      </c>
+      <c r="S4" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was wird mit wem gefeiert?'
+author: 'Nathan Gibson'
+session: 3
+tags: [3,slides]
+category: slides
+image: seder.jpg
+parallaxBackgroundImage: 'assets/img/seder.jpg'
+---
+</v>
+      </c>
+      <c r="T4" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Was wird mit wem gefeiert?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Die Rolle der schriftlichen und mündlichen "apostolischen" Traditionen im frühchristlichen Selbstverständnis skizzieren können. 
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Hybridität und Selbstpositionierung zwischen jüdischen Gemeinden und Jesu Nachfolger anhand von Ritualen illustrieren können.</v>
+      </c>
+      <c r="U4" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Warum ist es wichtig, richtig zu glauben?</v>
+      </c>
+      <c r="V4" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: 'Was wird mit wem gefeiert?'
+author: 'Nathan Gibson'
+session: 3
+tags: [3,slides]
+category: slides
+image: seder.jpg
+parallaxBackgroundImage: 'assets/img/seder.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Was wird mit wem gefeiert?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Die Rolle der schriftlichen und mündlichen "apostolischen" Traditionen im frühchristlichen Selbstverständnis skizzieren können. 
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Hybridität und Selbstpositionierung zwischen jüdischen Gemeinden und Jesu Nachfolger anhand von Ritualen illustrieren können.
+## Lektüre
+## Diskussion
+## Vorschau
+Warum ist es wichtig, richtig zu glauben?</v>
+      </c>
     </row>
-    <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
         <v>4</v>
       </c>
@@ -1273,8 +1571,78 @@
 level: overview
 ---</v>
       </c>
+      <c r="R5" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-05-19-4-slides.md</v>
+      </c>
+      <c r="S5" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Warum ist es wichtig, richtig zu glauben?'
+author: 'Nathan Gibson'
+session: 4
+tags: [4,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T5" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Warum ist es wichtig, richtig zu glauben?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Hybridität und Selbstpositionierung zwischen jüdischen Gemeinden und Jesu Nachfolger anhand von Ritualen illustrieren können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Sowohl die innere Logik der orthodoxischen Erzählung als auch historisch-kritische Bemerkungen daran erklären können.</v>
+      </c>
+      <c r="U5" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wer und was ist heilig?</v>
+      </c>
+      <c r="V5" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: 'Warum ist es wichtig, richtig zu glauben?'
+author: 'Nathan Gibson'
+session: 4
+tags: [4,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Warum ist es wichtig, richtig zu glauben?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Hybridität und Selbstpositionierung zwischen jüdischen Gemeinden und Jesu Nachfolger anhand von Ritualen illustrieren können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Sowohl die innere Logik der orthodoxischen Erzählung als auch historisch-kritische Bemerkungen daran erklären können.
+## Lektüre
+## Diskussion
+## Vorschau
+Wer und was ist heilig?</v>
+      </c>
     </row>
-    <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
         <v>5</v>
       </c>
@@ -1334,8 +1702,78 @@
 level: overview
 ---</v>
       </c>
+      <c r="R6" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-05-26-5-slides.md</v>
+      </c>
+      <c r="S6" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wer und was ist heilig?'
+author: 'Nathan Gibson'
+session: 5
+tags: [5,slides]
+category: slides
+image: aksehir-red-church-cappadocia.jpg
+parallaxBackgroundImage: 'assets/img/aksehir-red-church-cappadocia.jpg'
+---
+</v>
+      </c>
+      <c r="T6" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wer und was ist heilig?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Sowohl die innere Logik der orthodoxischen Erzählung als auch historisch-kritische Bemerkungen daran erklären können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Den Heiligkeitsbegriff mit Beispielen erklären können.</v>
+      </c>
+      <c r="U6" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie sieht eine Kirche aus?</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: 'Wer und was ist heilig?'
+author: 'Nathan Gibson'
+session: 5
+tags: [5,slides]
+category: slides
+image: aksehir-red-church-cappadocia.jpg
+parallaxBackgroundImage: 'assets/img/aksehir-red-church-cappadocia.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wer und was ist heilig?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Sowohl die innere Logik der orthodoxischen Erzählung als auch historisch-kritische Bemerkungen daran erklären können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Den Heiligkeitsbegriff mit Beispielen erklären können.
+## Lektüre
+## Diskussion
+## Vorschau
+Wie sieht eine Kirche aus?</v>
+      </c>
     </row>
-    <row r="7" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3">
         <v>6</v>
       </c>
@@ -1386,8 +1824,78 @@
 level: overview
 ---</v>
       </c>
+      <c r="R7" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-02-6-slides.md</v>
+      </c>
+      <c r="S7" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie sieht eine Kirche aus?'
+author: 'Nathan Gibson'
+session: 6
+tags: [6,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T7" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wie sieht eine Kirche aus?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Den Heiligkeitsbegriff mit Beispielen erklären können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.</v>
+      </c>
+      <c r="U7" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V7" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie sieht eine Kirche aus?'
+author: 'Nathan Gibson'
+session: 6
+tags: [6,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie sieht eine Kirche aus?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Den Heiligkeitsbegriff mit Beispielen erklären können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
     </row>
-    <row r="8" spans="1:17" s="11" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" s="11" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12"/>
       <c r="C8" s="13">
         <v>45817</v>
@@ -1405,8 +1913,77 @@
       </c>
       <c r="J8" s="12"/>
       <c r="M8" s="15"/>
+      <c r="R8" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-09-pfingstmontag-slides.md</v>
+      </c>
+      <c r="S8" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T8" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve"># Einführung ins Christentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U8" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie verstanden sich Christen und Muslime?</v>
+      </c>
+      <c r="V8" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+Wie verstanden sich Christen und Muslime?</v>
+      </c>
     </row>
-    <row r="9" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -1463,8 +2040,76 @@
 level: overview
 ---</v>
       </c>
+      <c r="R9" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-16-7-slides.md</v>
+      </c>
+      <c r="S9" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie verstanden sich Christen und Muslime?'
+author: 'Nathan Gibson'
+session: 7
+tags: [7,slides]
+category: slides
+image: st-paul-harissa.jpg
+parallaxBackgroundImage: 'assets/img/st-paul-harissa.jpg'
+---
+</v>
+      </c>
+      <c r="T9" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wie verstanden sich Christen und Muslime?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige Bereiche nennen können, in denen der langjährige Austausch zwischen islamischen und ostkirchlichen Gemeinschaften besonders bedeutsam war.</v>
+      </c>
+      <c r="U9" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
+      </c>
+      <c r="V9" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: 'Wie verstanden sich Christen und Muslime?'
+author: 'Nathan Gibson'
+session: 7
+tags: [7,slides]
+category: slides
+image: st-paul-harissa.jpg
+parallaxBackgroundImage: 'assets/img/st-paul-harissa.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie verstanden sich Christen und Muslime?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige Bereiche nennen können, in denen der langjährige Austausch zwischen islamischen und ostkirchlichen Gemeinschaften besonders bedeutsam war.
+## Lektüre
+## Diskussion
+## Vorschau
+Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
+      </c>
     </row>
-    <row r="10" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3">
         <v>8</v>
       </c>
@@ -1518,8 +2163,78 @@
 level: overview
 ---</v>
       </c>
+      <c r="R10" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-23-8-slides.md</v>
+      </c>
+      <c r="S10" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)'
+author: 'Nathan Gibson'
+session: 8
+tags: [8,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T10" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Bereiche nennen können, in denen der langjährige Austausch zwischen islamischen und ostkirchlichen Gemeinschaften besonders bedeutsam war.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Die größten Gemeinsamkeiten und Unterschiede zwischen der Kirche des Ostens und den griechischen oder römischen Kirchen identifizieren.</v>
+      </c>
+      <c r="U10" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
+      </c>
+      <c r="V10" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)'
+author: 'Nathan Gibson'
+session: 8
+tags: [8,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Bereiche nennen können, in denen der langjährige Austausch zwischen islamischen und ostkirchlichen Gemeinschaften besonders bedeutsam war.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Die größten Gemeinsamkeiten und Unterschiede zwischen der Kirche des Ostens und den griechischen oder römischen Kirchen identifizieren.
+## Lektüre
+## Diskussion
+## Vorschau
+Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
+      </c>
     </row>
-    <row r="11" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3">
         <v>9</v>
       </c>
@@ -1573,8 +2288,78 @@
 level: overview
 ---</v>
       </c>
+      <c r="R11" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-30-9-slides.md</v>
+      </c>
+      <c r="S11" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? '
+author: 'Nathan Gibson'
+session: 9
+tags: [9,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T11" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Die größten Gemeinsamkeiten und Unterschiede zwischen der Kirche des Ostens und den griechischen oder römischen Kirchen identifizieren.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.</v>
+      </c>
+      <c r="U11" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? '
+author: 'Nathan Gibson'
+session: 9
+tags: [9,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Die größten Gemeinsamkeiten und Unterschiede zwischen der Kirche des Ostens und den griechischen oder römischen Kirchen identifizieren.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
     </row>
-    <row r="12" spans="1:17" s="11" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" s="11" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12"/>
       <c r="C12" s="13">
         <v>45845</v>
@@ -1592,8 +2377,77 @@
       </c>
       <c r="J12" s="12"/>
       <c r="M12" s="15"/>
+      <c r="R12" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-09-sommerfest-slides.md</v>
+      </c>
+      <c r="S12" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T12" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve"># Einführung ins Christentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U12" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (II)</v>
+      </c>
+      <c r="V12" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (II)</v>
+      </c>
     </row>
-    <row r="13" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3">
         <v>10</v>
       </c>
@@ -1650,8 +2504,76 @@
 level: overview
 ---</v>
       </c>
+      <c r="R13" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-07-14-10-slides.md</v>
+      </c>
+      <c r="S13" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (II)'
+author: 'Nathan Gibson'
+session: 10
+tags: [10,slides]
+category: slides
+image: armenian-bell.jpg
+parallaxBackgroundImage: 'assets/img/armenian-bell.jpg'
+---
+</v>
+      </c>
+      <c r="T13" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (II)
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Eckpunkte der armenischen und äthiopischen Selbstnarrativen erzählen können.</v>
+      </c>
+      <c r="U13" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Was haben wir gelernt?</v>
+      </c>
+      <c r="V13" t="str">
+        <f t="shared" si="10"/>
+        <v>---
+layout: reveal
+title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (II)'
+author: 'Nathan Gibson'
+session: 10
+tags: [10,slides]
+category: slides
+image: armenian-bell.jpg
+parallaxBackgroundImage: 'assets/img/armenian-bell.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (II)
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Eckpunkte der armenischen und äthiopischen Selbstnarrativen erzählen können.
+## Lektüre
+## Diskussion
+## Vorschau
+Was haben wir gelernt?</v>
+      </c>
     </row>
-    <row r="14" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3">
         <v>11</v>
       </c>
@@ -1703,11 +2625,81 @@
 level: overview
 ---</v>
       </c>
+      <c r="R14" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-07-21-11-slides.md</v>
+      </c>
+      <c r="S14" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was haben wir gelernt?'
+author: 'Nathan Gibson'
+session: 11
+tags: [11,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T14" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve"># Einführung ins Christentum
+{: .r-fit-text}
+### Was haben wir gelernt?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Eckpunkte der armenischen und äthiopischen Selbstnarrativen erzählen können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Über die Kursinhalte reflektieren und das eingeworbene Wissen für sich versichern. </v>
+      </c>
+      <c r="U14" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V14" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was haben wir gelernt?'
+author: 'Nathan Gibson'
+session: 11
+tags: [11,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Was haben wir gelernt?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Eckpunkte der armenischen und äthiopischen Selbstnarrativen erzählen können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Über die Kursinhalte reflektieren und das eingeworbene Wissen für sich versichern. 
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E16" s="4"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rearranging sessions and images
</commit_message>
<xml_diff>
--- a/_data/sessions.xlsx
+++ b/_data/sessions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Github/jirelations/25christentum/_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46BB309-CA4C-4F44-A12E-0AB257F1170B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD17818-17A8-874E-AB68-09D6778A925F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4880" yWindow="500" windowWidth="46320" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sessions" sheetId="1" r:id="rId1"/>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="95">
   <si>
     <t>blank</t>
   </si>
@@ -548,6 +548,18 @@
   </si>
   <si>
     <t>tamckeIslamUndChristentum2008</t>
+  </si>
+  <si>
+    <t>coptic-incense.jpg</t>
+  </si>
+  <si>
+    <t>coptic-michael.jpg</t>
+  </si>
+  <si>
+    <t>bl-add-ms-7170-resurrection.jpg</t>
+  </si>
+  <si>
+    <t>wadi-qelt.jpg</t>
   </si>
 </sst>
 </file>
@@ -1991,7 +2003,7 @@
 ## Lektüre
 ## Diskussion
 ## Vorschau
-Wie sieht eine Kirche aus?</v>
+Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
       </c>
       <c r="V8" t="str">
         <f t="shared" si="10"/>
@@ -2019,7 +2031,7 @@
 ## Lektüre
 ## Diskussion
 ## Vorschau
-Wie sieht eine Kirche aus?</v>
+Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2034,29 +2046,37 @@
         <v>2025-06-16-7.md</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="I9" t="str">
         <f t="shared" si="4"/>
-        <v>7. Exkursion: Wie sieht eine Kirche aus?</v>
+        <v>7. Kirche des Ostens (ostsyrisch/assyrianisch): Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
       </c>
       <c r="J9" s="3">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
+      <c r="K9" t="s">
+        <v>93</v>
+      </c>
       <c r="L9" t="str">
         <f t="shared" si="5"/>
-        <v>7-Exkursion</v>
-      </c>
-      <c r="M9" s="16"/>
+        <v>7-Kirche-des-Ostens-(ostsyrisch/assyrianisch)</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N9" t="s">
-        <v>46</v>
+        <v>50</v>
+      </c>
+      <c r="O9" t="s">
+        <v>51</v>
       </c>
       <c r="P9" t="str">
         <f t="shared" si="2"/>
@@ -2076,16 +2096,26 @@
         <v>2025-06-16-7-slides.md</v>
       </c>
       <c r="S9" t="str">
-        <f t="shared" si="7"/>
+        <f>"---
+layout: reveal
+title: '"&amp;G9&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B9&amp;"
+tags: ["&amp;B9&amp;",slides]
+category: slides
+image: "&amp;K9&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K9&amp;"'
+---
+"</f>
         <v xml:space="preserve">---
 layout: reveal
-title: 'Wie sieht eine Kirche aus?'
+title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)'
 author: 'Nathan Gibson'
 session: 7
 tags: [7,slides]
 category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
+image: bl-add-ms-7170-resurrection.jpg
+parallaxBackgroundImage: 'assets/img/bl-add-ms-7170-resurrection.jpg'
 ---
 </v>
       </c>
@@ -2093,7 +2123,7 @@
         <f t="shared" si="8"/>
         <v># Einführung ins Christentum
 {: .r-fit-text}
-### Wie sieht eine Kirche aus?
+### Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)
 Sommersemester 2025
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
@@ -2101,7 +2131,7 @@
 ## Projekt
 ## Einleitung
 ## Heutiges Lernziel
-Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.</v>
+Die größten Gemeinsamkeiten und Unterschiede zwischen der Kirche des Ostens und den griechischen oder römischen Kirchen identifizieren.</v>
       </c>
       <c r="U9" t="str">
         <f t="shared" si="9"/>
@@ -2109,143 +2139,19 @@
 ## Lektüre
 ## Diskussion
 ## Vorschau
-Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
+Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
       </c>
       <c r="V9" t="str">
         <f t="shared" si="10"/>
-        <v>---
-layout: reveal
-title: 'Wie sieht eine Kirche aus?'
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)'
 author: 'Nathan Gibson'
 session: 7
 tags: [7,slides]
 category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
----
-# Einführung ins Christentum
-{: .r-fit-text}
-### Wie sieht eine Kirche aus?
-Sommersemester 2025
-Prof. Dr. Nathan Gibson
-## 📈 Rückblick: Lernziel
-## 📈 Rückblick: 
-## Projekt
-## Einleitung
-## Heutiges Lernziel
-Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
-## Lektüre
-## Diskussion
-## Vorschau
-Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="3">
-        <v>8</v>
-      </c>
-      <c r="C10" s="8">
-        <v>45831</v>
-      </c>
-      <c r="D10" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>2025-06-23-8.md</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G10" t="s">
-        <v>66</v>
-      </c>
-      <c r="I10" t="str">
-        <f t="shared" si="4"/>
-        <v>8. Kirche des Ostens (ostsyrisch/assyrianisch): Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)</v>
-      </c>
-      <c r="J10" s="3">
-        <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="L10" t="str">
-        <f t="shared" si="5"/>
-        <v>8-Kirche-des-Ostens-(ostsyrisch/assyrianisch)</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="N10" t="s">
-        <v>50</v>
-      </c>
-      <c r="O10" t="s">
-        <v>51</v>
-      </c>
-      <c r="P10" t="str">
-        <f t="shared" si="2"/>
-        <v>[8]</v>
-      </c>
-      <c r="Q10" t="str">
-        <f t="shared" si="3"/>
-        <v>---
-layout: post
-session: 8
-tags: [8]
-level: overview
----</v>
-      </c>
-      <c r="R10" t="str">
-        <f t="shared" si="6"/>
-        <v>2025-06-23-8-slides.md</v>
-      </c>
-      <c r="S10" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve">---
-layout: reveal
-title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)'
-author: 'Nathan Gibson'
-session: 8
-tags: [8,slides]
-category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
----
-</v>
-      </c>
-      <c r="T10" t="str">
-        <f t="shared" si="8"/>
-        <v># Einführung ins Christentum
-{: .r-fit-text}
-### Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)
-Sommersemester 2025
-Prof. Dr. Nathan Gibson
-## 📈 Rückblick: Lernziel
-Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
-## 📈 Rückblick: 
-## Projekt
-## Einleitung
-## Heutiges Lernziel
-Die größten Gemeinsamkeiten und Unterschiede zwischen der Kirche des Ostens und den griechischen oder römischen Kirchen identifizieren.</v>
-      </c>
-      <c r="U10" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve">
-## Lektüre
-## Diskussion
-## Vorschau
-Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
-      </c>
-      <c r="V10" t="str">
-        <f t="shared" si="10"/>
-        <v xml:space="preserve">---
-layout: reveal
-title: 'Wie entwickelte sich die Kirche außerhalb des Römischen Reiches? (I)'
-author: 'Nathan Gibson'
-session: 8
-tags: [8,slides]
-category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
+image: bl-add-ms-7170-resurrection.jpg
+parallaxBackgroundImage: 'assets/img/bl-add-ms-7170-resurrection.jpg'
 ---
 # Einführung ins Christentum
 {: .r-fit-text}
@@ -2253,7 +2159,6 @@
 Sommersemester 2025
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
-Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
 ## 📈 Rückblick: 
 ## Projekt
 ## Einleitung
@@ -2265,79 +2170,92 @@
 Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="3">
-        <v>9</v>
-      </c>
-      <c r="C11" s="8">
-        <v>45838</v>
-      </c>
-      <c r="D11" s="4" t="str">
+    <row r="10" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="3">
+        <v>8</v>
+      </c>
+      <c r="C10" s="8">
+        <v>45831</v>
+      </c>
+      <c r="D10" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>2025-06-30-9.md</v>
-      </c>
-      <c r="E11" s="4" t="s">
+        <v>2025-06-23-8.md</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G10" t="s">
         <v>68</v>
       </c>
-      <c r="I11" t="str">
+      <c r="I10" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">9. Kopten und Syrisch-Orthodoxen: Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
-      </c>
-      <c r="J11" s="3">
+        <v xml:space="preserve">8. Kopten und Syrisch-Orthodoxen: Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? </v>
+      </c>
+      <c r="J10" s="3">
         <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="L11" t="str">
+        <v>8</v>
+      </c>
+      <c r="K10" t="s">
+        <v>92</v>
+      </c>
+      <c r="L10" t="str">
         <f t="shared" si="5"/>
-        <v>9-Kopten-und-Syrisch-Orthodoxen</v>
-      </c>
-      <c r="M11" s="16" t="s">
+        <v>8-Kopten-und-Syrisch-Orthodoxen</v>
+      </c>
+      <c r="M10" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N10" t="s">
         <v>53</v>
       </c>
-      <c r="O11" t="s">
+      <c r="O10" t="s">
         <v>54</v>
       </c>
-      <c r="P11" t="str">
+      <c r="P10" t="str">
         <f t="shared" si="2"/>
-        <v>[9]</v>
-      </c>
-      <c r="Q11" t="str">
+        <v>[8]</v>
+      </c>
+      <c r="Q10" t="str">
         <f t="shared" si="3"/>
         <v>---
 layout: post
-session: 9
-tags: [9]
+session: 8
+tags: [8]
 level: overview
 ---</v>
       </c>
-      <c r="R11" t="str">
+      <c r="R10" t="str">
         <f t="shared" si="6"/>
-        <v>2025-06-30-9-slides.md</v>
-      </c>
-      <c r="S11" t="str">
-        <f t="shared" si="7"/>
+        <v>2025-06-23-8-slides.md</v>
+      </c>
+      <c r="S10" t="str">
+        <f>"---
+layout: reveal
+title: '"&amp;G10&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B10&amp;"
+tags: ["&amp;B10&amp;",slides]
+category: slides
+image: "&amp;K10&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K10&amp;"'
+---
+"</f>
         <v xml:space="preserve">---
 layout: reveal
 title: 'Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? '
 author: 'Nathan Gibson'
-session: 9
-tags: [9,slides]
-category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
+session: 8
+tags: [8,slides]
+category: slides
+image: coptic-michael.jpg
+parallaxBackgroundImage: 'assets/img/coptic-michael.jpg'
 ---
 </v>
       </c>
-      <c r="T11" t="str">
+      <c r="T10" t="str">
         <f t="shared" si="8"/>
         <v># Einführung ins Christentum
 {: .r-fit-text}
@@ -2352,25 +2270,25 @@
 ## Heutiges Lernziel
 Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.</v>
       </c>
-      <c r="U11" t="str">
+      <c r="U10" t="str">
         <f t="shared" si="9"/>
         <v xml:space="preserve">
 ## Lektüre
 ## Diskussion
 ## Vorschau
-</v>
-      </c>
-      <c r="V11" t="str">
+Wie sieht eine Kirche aus?</v>
+      </c>
+      <c r="V10" t="str">
         <f t="shared" si="10"/>
-        <v xml:space="preserve">---
+        <v>---
 layout: reveal
 title: 'Wie entfalteten sich die einheimischen Kirchen innerhalb des Römischen Reiches? '
 author: 'Nathan Gibson'
-session: 9
-tags: [9,slides]
-category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
+session: 8
+tags: [8,slides]
+category: slides
+image: coptic-michael.jpg
+parallaxBackgroundImage: 'assets/img/coptic-michael.jpg'
 ---
 # Einführung ins Christentum
 {: .r-fit-text}
@@ -2387,6 +2305,129 @@
 ## Lektüre
 ## Diskussion
 ## Vorschau
+Wie sieht eine Kirche aus?</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="3">
+        <v>9</v>
+      </c>
+      <c r="C11" s="8">
+        <v>45838</v>
+      </c>
+      <c r="D11" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>2025-06-30-9.md</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I11" t="str">
+        <f t="shared" si="4"/>
+        <v>9. Exkursion: Wie sieht eine Kirche aus?</v>
+      </c>
+      <c r="J11" s="3">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="K11" t="s">
+        <v>91</v>
+      </c>
+      <c r="L11" t="str">
+        <f t="shared" si="5"/>
+        <v>9-Exkursion</v>
+      </c>
+      <c r="M11" s="16"/>
+      <c r="N11" t="s">
+        <v>46</v>
+      </c>
+      <c r="P11" t="str">
+        <f t="shared" si="2"/>
+        <v>[9]</v>
+      </c>
+      <c r="Q11" t="str">
+        <f t="shared" si="3"/>
+        <v>---
+layout: post
+session: 9
+tags: [9]
+level: overview
+---</v>
+      </c>
+      <c r="R11" t="str">
+        <f t="shared" si="6"/>
+        <v>2025-06-30-9-slides.md</v>
+      </c>
+      <c r="S11" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie sieht eine Kirche aus?'
+author: 'Nathan Gibson'
+session: 9
+tags: [9,slides]
+category: slides
+image: coptic-incense.jpg
+parallaxBackgroundImage: 'assets/img/coptic-incense.jpg'
+---
+</v>
+      </c>
+      <c r="T11" t="str">
+        <f t="shared" si="8"/>
+        <v># Einführung ins Christentum
+{: .r-fit-text}
+### Wie sieht eine Kirche aus?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.</v>
+      </c>
+      <c r="U11" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie sieht eine Kirche aus?'
+author: 'Nathan Gibson'
+session: 9
+tags: [9,slides]
+category: slides
+image: coptic-incense.jpg
+parallaxBackgroundImage: 'assets/img/coptic-incense.jpg'
+---
+# Einführung ins Christentum
+{: .r-fit-text}
+### Wie sieht eine Kirche aus?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
+## Lektüre
+## Diskussion
+## Vorschau
 </v>
       </c>
     </row>
@@ -2434,7 +2475,7 @@
 Sommersemester 2025
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
-Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
 ## 📈 Rückblick: 
 ## Projekt
 ## Einleitung
@@ -2467,7 +2508,7 @@
 Sommersemester 2025
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
-Einige Aspekte der Identitätserzählung der koptischen und syrisch-orthodoxischen Gemeinden zusammenfassen können.
+Erfahren, wie in einer nicht-westlichen Tradition einen Gottesdienst gefeiert wird.
 ## 📈 Rückblick: 
 ## Projekt
 ## Einleitung
@@ -2632,6 +2673,9 @@
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
+      <c r="K14" t="s">
+        <v>94</v>
+      </c>
       <c r="L14" t="str">
         <f t="shared" si="5"/>
         <v>11-Rückblick</v>
@@ -2669,8 +2713,8 @@
 session: 11
 tags: [11,slides]
 category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
+image: wadi-qelt.jpg
+parallaxBackgroundImage: 'assets/img/wadi-qelt.jpg'
 ---
 </v>
       </c>
@@ -2706,8 +2750,8 @@
 session: 11
 tags: [11,slides]
 category: slides
-image: 
-parallaxBackgroundImage: 'assets/img/'
+image: wadi-qelt.jpg
+parallaxBackgroundImage: 'assets/img/wadi-qelt.jpg'
 ---
 # Einführung ins Christentum
 {: .r-fit-text}

</xml_diff>